<commit_message>
2026-06-15 Catchup for Hockey Pool, NHL Scoreboard, Job Hunt, Resource, Thingiverse
</commit_message>
<xml_diff>
--- a/Python/Hockey pool/2024/My Predictions.xlsx
+++ b/Python/Hockey pool/2024/My Predictions.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
-  <workbookPr defaultThemeVersion="166925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abrig\Documents\Coding_Practice\Python\Hockey pool\2024\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F6844C5-05D0-4916-A277-27353F956372}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EF88D4F-29FD-40E5-B133-F2FAB661A4BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{7BF13B1A-4770-4E31-9A10-40459726CAB5}"/>
   </bookViews>
@@ -1468,6 +1468,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0969FCB-44D6-4DD7-80C6-C6E6D39A1DF9}">
+  <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:CE90"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>